<commit_message>
IMPORTANT CHANGES: (1): Got GradCAM working for GoogLeNet without pretraining; (2): Commented out unused gradCAM code. Minor changes: (1) Ensured plots are closed at the end of functions, (2) set net to eval in gradCAM function (although this is unncessary since it is already set to eval in object
</commit_message>
<xml_diff>
--- a/Results/Study 1/GoogLeNet (pretrained)/Confusion Matrices.xlsx
+++ b/Results/Study 1/GoogLeNet (pretrained)/Confusion Matrices.xlsx
@@ -400,10 +400,10 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>508</v>
+        <v>495</v>
       </c>
       <c r="C2">
-        <v>132</v>
+        <v>145</v>
       </c>
     </row>
     <row r="3" spans="1:3">
@@ -411,10 +411,10 @@
         <v>3</v>
       </c>
       <c r="B3">
-        <v>213</v>
+        <v>218</v>
       </c>
       <c r="C3">
-        <v>427</v>
+        <v>422</v>
       </c>
     </row>
   </sheetData>

</xml_diff>